<commit_message>
Update daily Zee Business signals
</commit_message>
<xml_diff>
--- a/zeebiz_live_stocks.xlsx
+++ b/zeebiz_live_stocks.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Latest by Stock" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Website Signals'!$A$1:$J$1490</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Website Signals'!$A$1:$J$1562</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Latest by Stock'!$A$1:$J$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1490"/>
+  <dimension ref="A1:J1562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -56464,11 +56464,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1328" t="inlineStr"/>
       <c r="E1328" t="n">
         <v>9235</v>
       </c>
-      <c r="G1328" t="inlineStr"/>
       <c r="H1328" t="inlineStr">
         <is>
           <t>Divi's Lab Fut 9548.00 222.00 BUY TARGET HIT 9235</t>
@@ -56501,14 +56499,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1329" t="inlineStr"/>
       <c r="E1329" t="n">
         <v>9480</v>
       </c>
       <c r="F1329" t="n">
         <v>9235</v>
       </c>
-      <c r="G1329" t="inlineStr"/>
       <c r="H1329" t="inlineStr">
         <is>
           <t>Divi's Lab Fut 9548.00 222.00 BUY TGT 9480 SL 9235</t>
@@ -56541,14 +56537,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1330" t="inlineStr"/>
       <c r="E1330" t="n">
         <v>9480</v>
       </c>
       <c r="F1330" t="n">
         <v>9235</v>
       </c>
-      <c r="G1330" t="inlineStr"/>
       <c r="H1330" t="inlineStr">
         <is>
           <t>Divi's Lab Fut 9548.00 2.38% BUY TGT 9480 SL 9235</t>
@@ -56581,11 +56575,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1331" t="inlineStr"/>
       <c r="E1331" t="n">
         <v>9480</v>
       </c>
-      <c r="G1331" t="inlineStr"/>
       <c r="H1331" t="inlineStr">
         <is>
           <t>Divi's Lab Fut 9548.00 222.00 BUY TGT 9480</t>
@@ -56624,7 +56616,6 @@
       <c r="E1332" t="n">
         <v>8600</v>
       </c>
-      <c r="G1332" t="inlineStr"/>
       <c r="H1332" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -56671,7 +56662,6 @@
       <c r="F1333" t="n">
         <v>161</v>
       </c>
-      <c r="G1333" t="inlineStr"/>
       <c r="H1333" t="inlineStr">
         <is>
           <t>सुमित के सुपरहिट Bandhan Bank 171.30 6.60 BUY TGT 175 SL 161</t>
@@ -56710,7 +56700,6 @@
       <c r="E1334" t="n">
         <v>175</v>
       </c>
-      <c r="G1334" t="inlineStr"/>
       <c r="H1334" t="inlineStr">
         <is>
           <t>Bandhan Bank 171.37 ▲ 6.67 BUY TGT 175</t>
@@ -56749,7 +56738,6 @@
       <c r="E1335" t="n">
         <v>535</v>
       </c>
-      <c r="G1335" t="inlineStr"/>
       <c r="H1335" t="inlineStr">
         <is>
           <t>Hind Copper 532.45 4.63% BUY TGT 535 DUR 6 महीने</t>
@@ -56791,7 +56779,6 @@
       <c r="F1336" t="n">
         <v>999</v>
       </c>
-      <c r="G1336" t="inlineStr"/>
       <c r="H1336" t="inlineStr">
         <is>
           <t>सुमित के सुपरहिट Hindalco 1018.80 12.80 BUY TGT 1040 SL 999</t>
@@ -56824,7 +56811,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1337" t="inlineStr"/>
       <c r="E1337" t="n">
         <v>930</v>
       </c>
@@ -56865,7 +56851,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1338" t="inlineStr"/>
       <c r="E1338" t="n">
         <v>730</v>
       </c>
@@ -56906,14 +56891,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1339" t="inlineStr"/>
       <c r="E1339" t="n">
         <v>990</v>
       </c>
       <c r="F1339" t="n">
         <v>930</v>
       </c>
-      <c r="G1339" t="inlineStr"/>
       <c r="H1339" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Jubilant Pharmova 1011.20 6.41% BUY TGT 990 SL 930</t>
@@ -56955,7 +56938,6 @@
       <c r="F1340" t="n">
         <v>1890</v>
       </c>
-      <c r="G1340" t="inlineStr"/>
       <c r="H1340" t="inlineStr">
         <is>
           <t>11 बजे की लेडीज स्पेशल
@@ -56993,7 +56975,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1341" t="inlineStr"/>
       <c r="E1341" t="n">
         <v>6000</v>
       </c>
@@ -57086,7 +57067,6 @@
       <c r="E1343" t="n">
         <v>6000</v>
       </c>
-      <c r="G1343" t="inlineStr"/>
       <c r="H1343" t="inlineStr">
         <is>
           <t>BUZZING STOCK GE Vernova T&amp;D 4739.00 ▲ 8.51% खरीदारी की राश, लक्ष्य ₹5675 से बढ़ाकर ₹6000</t>
@@ -57119,14 +57099,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1344" t="inlineStr"/>
       <c r="E1344" t="n">
         <v>9480</v>
       </c>
       <c r="F1344" t="n">
         <v>9235</v>
       </c>
-      <c r="G1344" t="inlineStr"/>
       <c r="H1344" t="inlineStr">
         <is>
           <t>जय का JACKPOT
@@ -57164,11 +57142,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1345" t="inlineStr"/>
       <c r="E1345" t="n">
         <v>9480</v>
       </c>
-      <c r="G1345" t="inlineStr"/>
       <c r="H1345" t="inlineStr">
         <is>
           <t>Divi's Lab Fut 9514.50 188.50 BUY TGT 9480</t>
@@ -57201,14 +57177,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1346" t="inlineStr"/>
       <c r="E1346" t="n">
         <v>425</v>
       </c>
       <c r="F1346" t="n">
         <v>408</v>
       </c>
-      <c r="G1346" t="inlineStr"/>
       <c r="H1346" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर
@@ -57255,7 +57229,6 @@
       <c r="F1347" t="n">
         <v>161</v>
       </c>
-      <c r="G1347" t="inlineStr"/>
       <c r="H1347" t="inlineStr">
         <is>
           <t>सुमीत के सुपरहिट
@@ -57302,7 +57275,6 @@
       <c r="F1348" t="n">
         <v>999</v>
       </c>
-      <c r="G1348" t="inlineStr"/>
       <c r="H1348" t="inlineStr">
         <is>
           <t>Hindalco 1022.00 16.00 BUY TGT 1040 SL 999</t>
@@ -57344,7 +57316,6 @@
       <c r="F1349" t="n">
         <v>728</v>
       </c>
-      <c r="G1349" t="inlineStr"/>
       <c r="H1349" t="inlineStr">
         <is>
           <t>SHORT MIDCAP STOCKS TD Power खरीदें STOP LOSS 728 TARGET 810/830 DURATION -- TD Power 769.00</t>
@@ -57432,7 +57403,6 @@
       <c r="F1351" t="n">
         <v>215</v>
       </c>
-      <c r="G1351" t="inlineStr"/>
       <c r="H1351" t="inlineStr">
         <is>
           <t>संदीप जैन की राय South West Pinnacle खरीदें STOP LOSS 215 TARGET 240/245 DURATION -- South West Pinnacle 222.67 ▲ 0.18%</t>
@@ -57474,7 +57444,6 @@
       <c r="F1352" t="n">
         <v>215</v>
       </c>
-      <c r="G1352" t="inlineStr"/>
       <c r="H1352" t="inlineStr">
         <is>
           <t>संदीप जैन की राय South West Pinnacle खरीदें STOP LOSS 215 TARGET 240/245 DURATION -- South West Pinnacle 222.67 ▲ 0.18%</t>
@@ -57507,14 +57476,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1353" t="inlineStr"/>
       <c r="E1353" t="n">
         <v>250</v>
       </c>
       <c r="F1353" t="n">
         <v>218</v>
       </c>
-      <c r="G1353" t="inlineStr"/>
       <c r="H1353" t="inlineStr">
         <is>
           <t>POSITIONAL MIDCAP STOCK BHARAT SEATS LIMITED खरीदें STOP LOSS 218 TARGET 250/255 DURATION</t>
@@ -57547,14 +57514,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1354" t="inlineStr"/>
       <c r="E1354" t="n">
         <v>255</v>
       </c>
       <c r="F1354" t="n">
         <v>218</v>
       </c>
-      <c r="G1354" t="inlineStr"/>
       <c r="H1354" t="inlineStr">
         <is>
           <t>POSITIONAL MIDCAP STOCK BHARAT SEATS LIMITED खरीदें STOP LOSS 218 TARGET 250/255 DURATION</t>
@@ -57587,14 +57552,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1355" t="inlineStr"/>
       <c r="E1355" t="n">
         <v>158</v>
       </c>
       <c r="F1355" t="n">
         <v>132</v>
       </c>
-      <c r="G1355" t="inlineStr"/>
       <c r="H1355" t="inlineStr">
         <is>
           <t>TN Petro खरीदें PRICE 143.57 TARGET 158/170 STOP LOSS 132</t>
@@ -57636,7 +57599,6 @@
       <c r="F1356" t="n">
         <v>406</v>
       </c>
-      <c r="G1356" t="inlineStr"/>
       <c r="H1356" t="inlineStr">
         <is>
           <t>BEL Fut 417.50 11.15 BUY TGT 418 SL 406</t>
@@ -57675,7 +57637,6 @@
       <c r="E1357" t="n">
         <v>1950</v>
       </c>
-      <c r="G1357" t="inlineStr"/>
       <c r="H1357" t="inlineStr">
         <is>
           <t>जैन साब के GEMS Astra Micro 1745.50 33.90 BUY TGT 1950 SL --</t>
@@ -57717,7 +57678,6 @@
       <c r="F1358" t="n">
         <v>161</v>
       </c>
-      <c r="G1358" t="inlineStr"/>
       <c r="H1358" t="inlineStr">
         <is>
           <t>Bandhan Bank 170.45 5.75 BUY TGT 175 SL 161</t>
@@ -57759,7 +57719,6 @@
       <c r="F1359" t="n">
         <v>4580</v>
       </c>
-      <c r="G1359" t="inlineStr"/>
       <c r="H1359" t="inlineStr">
         <is>
           <t>POSITIONAL MIDCAP STOCKS
@@ -57805,7 +57764,6 @@
       <c r="F1360" t="n">
         <v>4580</v>
       </c>
-      <c r="G1360" t="inlineStr"/>
       <c r="H1360" t="inlineStr">
         <is>
           <t>CRISIL खरीदें STOP LOSS 4580 TARGET 5100/5150 DURATION -- CRISIL 4799.90 13.30</t>
@@ -57844,7 +57802,6 @@
       <c r="E1361" t="n">
         <v>421</v>
       </c>
-      <c r="G1361" t="inlineStr"/>
       <c r="H1361" t="inlineStr">
         <is>
           <t>SUPER SID BEL 415.10 11.10 BUY TGT 421 DUR 6 महीने</t>
@@ -57877,11 +57834,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1362" t="inlineStr"/>
       <c r="E1362" t="n">
         <v>535</v>
       </c>
-      <c r="G1362" t="inlineStr"/>
       <c r="H1362" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -57928,7 +57883,6 @@
       <c r="F1363" t="n">
         <v>999</v>
       </c>
-      <c r="G1363" t="inlineStr"/>
       <c r="H1363" t="inlineStr">
         <is>
           <t>Hindalco 1023.40 17.40 BUY TGT 1040 SL 999</t>
@@ -57967,7 +57921,6 @@
       <c r="E1364" t="n">
         <v>1040</v>
       </c>
-      <c r="G1364" t="inlineStr"/>
       <c r="H1364" t="inlineStr">
         <is>
           <t>Hindalco 1023.00 17.00 BUY TGT 1040</t>
@@ -58009,7 +57962,6 @@
       <c r="F1365" t="n">
         <v>218</v>
       </c>
-      <c r="G1365" t="inlineStr"/>
       <c r="H1365" t="inlineStr">
         <is>
           <t>POSITIONAL MIDCAP STOCKS
@@ -58057,7 +58009,6 @@
       <c r="F1366" t="n">
         <v>218</v>
       </c>
-      <c r="G1366" t="inlineStr"/>
       <c r="H1366" t="inlineStr">
         <is>
           <t>BHARAT SEATS LIMITED खरीदें STOP LOSS 218 TARGET 250/255 DURATION -- Bharat Seats Ltd 225.63</t>
@@ -58096,7 +58047,6 @@
       <c r="E1367" t="n">
         <v>1430</v>
       </c>
-      <c r="G1367" t="inlineStr"/>
       <c r="H1367" t="inlineStr">
         <is>
           <t>LONG MIDCAP STOCKS Aegis Logistics खरीदें STOP LOSS -- TARGET 1430/1450 DURATION 6-12 महीने Aegis Logistics 1247.20 6.50</t>
@@ -58135,7 +58085,6 @@
       <c r="E1368" t="n">
         <v>1450</v>
       </c>
-      <c r="G1368" t="inlineStr"/>
       <c r="H1368" t="inlineStr">
         <is>
           <t>LONG MIDCAP STOCKS Aegis Logistics खरीदें STOP LOSS -- TARGET 1430/1450 DURATION 6-12 महीने Aegis Logistics 1247.20 6.50</t>
@@ -58174,7 +58123,6 @@
       <c r="E1369" t="n">
         <v>1430</v>
       </c>
-      <c r="G1369" t="inlineStr"/>
       <c r="H1369" t="inlineStr">
         <is>
           <t>सदीप जैन का राय Aegis Logistics खरीदें STOP LOSS -- TARGET 1430/1450 DURATION 6-12 महीने Aegis Logistics 1246.90 0.54%</t>
@@ -58213,7 +58161,6 @@
       <c r="E1370" t="n">
         <v>1450</v>
       </c>
-      <c r="G1370" t="inlineStr"/>
       <c r="H1370" t="inlineStr">
         <is>
           <t>संदीप जैन की राय Aegis Logistics खरीदें STOP LOSS -- TARGET 1430/1450 DURATION 6-12 महीने Aegis Logistics 1246.90</t>
@@ -58338,14 +58285,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1373" t="inlineStr"/>
       <c r="E1373" t="n">
         <v>420</v>
       </c>
       <c r="F1373" t="n">
         <v>280</v>
       </c>
-      <c r="G1373" t="inlineStr"/>
       <c r="H1373" t="inlineStr">
         <is>
           <t>Prime Focus खरीदें PRICE 321.10 TARGET 420/450 STOP LOSS 280</t>
@@ -58387,7 +58332,6 @@
       <c r="F1374" t="n">
         <v>280</v>
       </c>
-      <c r="G1374" t="inlineStr"/>
       <c r="H1374" t="inlineStr">
         <is>
           <t>1 की कमाई Prime Focus खरीदें PRICE 320.90 TARGET 420/450 STOP LOSS 280</t>
@@ -58429,7 +58373,6 @@
       <c r="F1375" t="n">
         <v>280</v>
       </c>
-      <c r="G1375" t="inlineStr"/>
       <c r="H1375" t="inlineStr">
         <is>
           <t>Prime Focus खरीदें PRICE 321.10 TARGET 420/450 STOP LOSS 280</t>
@@ -58468,7 +58411,6 @@
       <c r="E1376" t="n">
         <v>8600</v>
       </c>
-      <c r="G1376" t="inlineStr"/>
       <c r="H1376" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -58515,7 +58457,6 @@
       <c r="F1377" t="n">
         <v>406</v>
       </c>
-      <c r="G1377" t="inlineStr"/>
       <c r="H1377" t="inlineStr">
         <is>
           <t>BEL Fut 416.00 9.65 BUY TGT 418 SL 406</t>
@@ -58554,7 +58495,6 @@
       <c r="E1378" t="n">
         <v>1950</v>
       </c>
-      <c r="G1378" t="inlineStr"/>
       <c r="H1378" t="inlineStr">
         <is>
           <t>जैन साब के GEMS
@@ -58598,7 +58538,6 @@
       <c r="E1379" t="n">
         <v>421</v>
       </c>
-      <c r="G1379" t="inlineStr"/>
       <c r="H1379" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -58642,7 +58581,6 @@
       <c r="E1380" t="n">
         <v>421</v>
       </c>
-      <c r="G1380" t="inlineStr"/>
       <c r="H1380" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -58686,7 +58624,6 @@
       <c r="E1381" t="n">
         <v>535</v>
       </c>
-      <c r="G1381" t="inlineStr"/>
       <c r="H1381" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -58733,7 +58670,6 @@
       <c r="F1382" t="n">
         <v>999</v>
       </c>
-      <c r="G1382" t="inlineStr"/>
       <c r="H1382" t="inlineStr">
         <is>
           <t>Hindalco 1020.70 14.70 BUY TGT 1040 SL 999</t>
@@ -58852,11 +58788,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1385" t="inlineStr"/>
       <c r="E1385" t="n">
         <v>3880</v>
       </c>
-      <c r="G1385" t="inlineStr"/>
       <c r="H1385" t="inlineStr">
         <is>
           <t>SUPER SID Sansera Engg 4034.40 BUY TGT 3880 TARGET HIT</t>
@@ -58895,7 +58829,6 @@
       <c r="E1386" t="n">
         <v>4172.5</v>
       </c>
-      <c r="G1386" t="inlineStr"/>
       <c r="H1386" t="inlineStr">
         <is>
           <t>SUPER SID Sansera Engg 4034.40 138.10 BUY TARGET HIT</t>
@@ -58928,11 +58861,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1387" t="inlineStr"/>
       <c r="E1387" t="n">
         <v>3990</v>
       </c>
-      <c r="G1387" t="inlineStr"/>
       <c r="H1387" t="inlineStr">
         <is>
           <t>SUPER SID Sansera Engg 4034.40 138.10 BUY TGT 3990 SL</t>
@@ -58965,11 +58896,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1388" t="inlineStr"/>
       <c r="E1388" t="n">
         <v>3980</v>
       </c>
-      <c r="G1388" t="inlineStr"/>
       <c r="H1388" t="inlineStr">
         <is>
           <t>Sansera Engg 4031.60 135.30 BUY TGT 3980 SL --</t>
@@ -59011,7 +58940,6 @@
       <c r="F1389" t="n">
         <v>408</v>
       </c>
-      <c r="G1389" t="inlineStr"/>
       <c r="H1389" t="inlineStr">
         <is>
           <t>विशेष के विशेष BEL Fut 414.95 9.88 BUY TGT 418 SL 408</t>
@@ -59050,7 +58978,6 @@
       <c r="E1390" t="n">
         <v>418</v>
       </c>
-      <c r="G1390" t="inlineStr"/>
       <c r="H1390" t="inlineStr">
         <is>
           <t>BEL Fut 415.10 8.75 BUY TGT 418</t>
@@ -59083,14 +59010,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1391" t="inlineStr"/>
       <c r="E1391" t="n">
         <v>250</v>
       </c>
       <c r="F1391" t="n">
         <v>150</v>
       </c>
-      <c r="G1391" t="inlineStr"/>
       <c r="H1391" t="inlineStr">
         <is>
           <t>सुमित बगडिया की राय DIVI'S LAB 9400 की कॉल @ ₹191 खरीदें STOP LOSS 150 TARGET 250/280 Divi's Lab 9400.00 ▲ 1.02%</t>
@@ -59123,14 +59048,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1392" t="inlineStr"/>
       <c r="E1392" t="n">
         <v>280</v>
       </c>
       <c r="F1392" t="n">
         <v>150</v>
       </c>
-      <c r="G1392" t="inlineStr"/>
       <c r="H1392" t="inlineStr">
         <is>
           <t>सुमित बगडिया की राय DIVI'S LAB 9400 की कॉल @ ₹191 खरीदें STOP LOSS 150 TARGET 250/280 Divi's Lab 9400.00 ▲ 1.02%</t>
@@ -59163,14 +59086,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1393" t="inlineStr"/>
       <c r="E1393" t="n">
         <v>425</v>
       </c>
       <c r="F1393" t="n">
         <v>408</v>
       </c>
-      <c r="G1393" t="inlineStr"/>
       <c r="H1393" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर
@@ -59213,7 +59134,6 @@
       <c r="E1394" t="n">
         <v>535</v>
       </c>
-      <c r="G1394" t="inlineStr"/>
       <c r="H1394" t="inlineStr">
         <is>
           <t>SUPER SID Hind Copper 529.30 4.01% BUY TGT 535 BUR ₹ नहीं</t>
@@ -59246,11 +59166,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1395" t="inlineStr"/>
       <c r="E1395" t="n">
         <v>51.15</v>
       </c>
-      <c r="G1395" t="inlineStr"/>
       <c r="H1395" t="inlineStr">
         <is>
           <t>DIVISLAB 9400 CALL ▲
@@ -59297,7 +59215,6 @@
       <c r="F1396" t="n">
         <v>999</v>
       </c>
-      <c r="G1396" t="inlineStr"/>
       <c r="H1396" t="inlineStr">
         <is>
           <t>सुमीत के सुपरहिट Hindalco 1015.30 9.30 BUY TGT 1040 SL 999</t>
@@ -59330,11 +59247,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1397" t="inlineStr"/>
       <c r="E1397" t="n">
         <v>4705</v>
       </c>
-      <c r="G1397" t="inlineStr"/>
       <c r="H1397" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर Data Patterns 4798.90 4.53% BUY TARGET HIT 4705</t>
@@ -59367,11 +59282,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1398" t="inlineStr"/>
       <c r="E1398" t="n">
         <v>50</v>
       </c>
-      <c r="G1398" t="inlineStr"/>
       <c r="H1398" t="inlineStr">
         <is>
           <t>DIVISLAB 9400 CALL ▲ 203.65 ▲ 50.00 32.54% EXPIRY- 29 SEP 2026 OPEN INTEREST 1.08 Lk ▲ 0.12 Lk Divi's Lab 9402.50 87.50</t>
@@ -59404,11 +59317,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1399" t="inlineStr"/>
       <c r="E1399" t="n">
         <v>4705</v>
       </c>
-      <c r="G1399" t="inlineStr"/>
       <c r="H1399" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर Data Patterns 4799.80 4.55% BUY TARGET HIT 4705</t>
@@ -59441,14 +59352,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1400" t="inlineStr"/>
       <c r="E1400" t="n">
         <v>4800</v>
       </c>
       <c r="F1400" t="n">
         <v>4705</v>
       </c>
-      <c r="G1400" t="inlineStr"/>
       <c r="H1400" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर Data Patterns 4803.50 212.70 BUY TGT 4800 SL 4705</t>
@@ -59481,14 +59390,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1401" t="inlineStr"/>
       <c r="E1401" t="n">
         <v>4800</v>
       </c>
       <c r="F1401" t="n">
         <v>4705</v>
       </c>
-      <c r="G1401" t="inlineStr"/>
       <c r="H1401" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर Data Patterns 4801.10 210.30 BUY TGT 4800 SL 4705</t>
@@ -59650,14 +59557,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1405" t="inlineStr"/>
       <c r="E1405" t="n">
         <v>421</v>
       </c>
       <c r="F1405" t="n">
         <v>500</v>
       </c>
-      <c r="G1405" t="inlineStr"/>
       <c r="H1405" t="inlineStr">
         <is>
           <t>BEL खरीदें PRICE 412.45 TARGET 421/500 DURATION 6 महीने</t>
@@ -59785,7 +59690,6 @@
       <c r="F1408" t="n">
         <v>406</v>
       </c>
-      <c r="G1408" t="inlineStr"/>
       <c r="H1408" t="inlineStr">
         <is>
           <t>विशेष चौहान की राय BEL Fut खरीदें PRICE 413.60 TARGET 418/426 STOP LOSS 406</t>
@@ -59827,7 +59731,6 @@
       <c r="F1409" t="n">
         <v>406</v>
       </c>
-      <c r="G1409" t="inlineStr"/>
       <c r="H1409" t="inlineStr">
         <is>
           <t>विशेष चौहान की राय BEL Fut खरीदें PRICE 413.60 TARGET 418/426 STOP LOSS 406</t>
@@ -59866,7 +59769,6 @@
       <c r="E1410" t="n">
         <v>426</v>
       </c>
-      <c r="G1410" t="inlineStr"/>
       <c r="H1410" t="inlineStr">
         <is>
           <t>BEL Fut PRICE 413.55 TARGET 418/426</t>
@@ -59905,7 +59807,6 @@
       <c r="E1411" t="n">
         <v>1990</v>
       </c>
-      <c r="G1411" t="inlineStr"/>
       <c r="H1411" t="inlineStr">
         <is>
           <t>Astra Micro खरीदें PRICE 1742.00 TARGET 1950/1990 STOP LOSS --</t>
@@ -59944,7 +59845,6 @@
       <c r="E1412" t="n">
         <v>1950</v>
       </c>
-      <c r="G1412" t="inlineStr"/>
       <c r="H1412" t="inlineStr">
         <is>
           <t>Astra Micro खरीदें PRICE 1742.00 TARGET 1950/1990 STOP LOSS --</t>
@@ -59983,7 +59883,6 @@
       <c r="E1413" t="n">
         <v>1950</v>
       </c>
-      <c r="G1413" t="inlineStr"/>
       <c r="H1413" t="inlineStr">
         <is>
           <t>जन साब के GEMS
@@ -60027,7 +59926,6 @@
       <c r="E1414" t="n">
         <v>1990</v>
       </c>
-      <c r="G1414" t="inlineStr"/>
       <c r="H1414" t="inlineStr">
         <is>
           <t>जन साब के GEMS
@@ -60074,7 +59972,6 @@
       <c r="F1415" t="n">
         <v>232</v>
       </c>
-      <c r="G1415" t="inlineStr"/>
       <c r="H1415" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर Data Patterns 4822.80 232.00 BUY</t>
@@ -60107,14 +60004,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1416" t="inlineStr"/>
       <c r="E1416" t="n">
         <v>4800</v>
       </c>
       <c r="F1416" t="n">
         <v>4705</v>
       </c>
-      <c r="G1416" t="inlineStr"/>
       <c r="H1416" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर Data Patterns 4822.00 231.20 BUY TGT 4800 SL 4705</t>
@@ -60147,14 +60042,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1417" t="inlineStr"/>
       <c r="E1417" t="n">
         <v>4800</v>
       </c>
       <c r="F1417" t="n">
         <v>4705</v>
       </c>
-      <c r="G1417" t="inlineStr"/>
       <c r="H1417" t="inlineStr">
         <is>
           <t>Astra Micro 1747.50 TODAY 1783 HIGH 1783.30 LOW 1708.30 Vol: 263.96 k शुभ 'मंगला' शेयर Data Patterns 4819.40 4.98% BUY TGT 4800 SL 4705</t>
@@ -60187,14 +60080,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1418" t="inlineStr"/>
       <c r="E1418" t="n">
         <v>425</v>
       </c>
       <c r="F1418" t="n">
         <v>408</v>
       </c>
-      <c r="G1418" t="inlineStr"/>
       <c r="H1418" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर LIC खरीदें PRICE 415.25 TARGET 425/435 STOP LOSS 408</t>
@@ -60227,14 +60118,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1419" t="inlineStr"/>
       <c r="E1419" t="n">
         <v>435</v>
       </c>
       <c r="F1419" t="n">
         <v>408</v>
       </c>
-      <c r="G1419" t="inlineStr"/>
       <c r="H1419" t="inlineStr">
         <is>
           <t>शुभ 'मंगला' शेयर LIC खरीदें PRICE 415.25 TARGET 425/435 STOP LOSS 408</t>
@@ -60273,7 +60162,6 @@
       <c r="E1420" t="n">
         <v>4100.9</v>
       </c>
-      <c r="G1420" t="inlineStr"/>
       <c r="H1420" t="inlineStr">
         <is>
           <t>SUPER SID Sansera Engg 3997.60 101.30 BUY TARGET HIT</t>
@@ -60312,7 +60200,6 @@
       <c r="E1421" t="n">
         <v>535</v>
       </c>
-      <c r="G1421" t="inlineStr"/>
       <c r="H1421" t="inlineStr">
         <is>
           <t>SUPER SID
@@ -60359,7 +60246,6 @@
       <c r="F1422" t="n">
         <v>4705</v>
       </c>
-      <c r="G1422" t="inlineStr"/>
       <c r="H1422" t="inlineStr">
         <is>
           <t>Data Patterns 4785.00 4.23% BUY TGT 4800 SL 4705</t>
@@ -60392,14 +60278,12 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1423" t="inlineStr"/>
       <c r="E1423" t="n">
         <v>4800</v>
       </c>
       <c r="F1423" t="n">
         <v>4705</v>
       </c>
-      <c r="G1423" t="inlineStr"/>
       <c r="H1423" t="inlineStr">
         <is>
           <t>Intellect Design 683.70 ▲ 0.23% HIGH 688.00 LOW 677.00 Vol: 34.54 k शुभ 'मंगला' शेयर Data Patterns 4784.00 BUY TGT 4800 SL 4705</t>
@@ -60441,7 +60325,6 @@
       <c r="F1424" t="n">
         <v>161</v>
       </c>
-      <c r="G1424" t="inlineStr"/>
       <c r="H1424" t="inlineStr">
         <is>
           <t>सुमित बगडिया की राय Bandhan Bank खरीदें PRICE 167.80 TARGET 175/184 STOP LOSS 161</t>
@@ -60483,7 +60366,6 @@
       <c r="F1425" t="n">
         <v>161</v>
       </c>
-      <c r="G1425" t="inlineStr"/>
       <c r="H1425" t="inlineStr">
         <is>
           <t>सुमित बगडिया की राय Bandhan Bank खरीदें PRICE 167.80 TARGET 175/184 STOP LOSS 161</t>
@@ -60565,7 +60447,6 @@
       <c r="E1427" t="n">
         <v>500</v>
       </c>
-      <c r="G1427" t="inlineStr"/>
       <c r="H1427" t="inlineStr">
         <is>
           <t>BEL खरीदें PRICE 409.20 TARGET 421/500 DURATION 6 महीने</t>
@@ -60604,7 +60485,6 @@
       <c r="E1428" t="n">
         <v>500</v>
       </c>
-      <c r="G1428" t="inlineStr"/>
       <c r="H1428" t="inlineStr">
         <is>
           <t>SUPER SID BEL खरीदें PRICE 409.10 TARGET 421/500 DURATION 6 महीने</t>
@@ -60680,11 +60560,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1430" t="inlineStr"/>
       <c r="E1430" t="n">
         <v>3998</v>
       </c>
-      <c r="G1430" t="inlineStr"/>
       <c r="H1430" t="inlineStr">
         <is>
           <t>SID Sansera Engg 4641.00 BUY 3998 TARGET HIT</t>
@@ -60717,11 +60595,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1431" t="inlineStr"/>
       <c r="E1431" t="n">
         <v>327.25</v>
       </c>
-      <c r="G1431" t="inlineStr"/>
       <c r="H1431" t="inlineStr">
         <is>
           <t>PCBL Chemical 327.25 INVESTMENT PICK 264.00 11/07/2024 RECO PRICE RETURN TILL NOW 63.25 23.96%</t>
@@ -60754,11 +60630,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1432" t="inlineStr"/>
       <c r="E1432" t="n">
         <v>4024.3</v>
       </c>
-      <c r="G1432" t="inlineStr"/>
       <c r="H1432" t="inlineStr">
         <is>
           <t>Sansera Engg 4024.30 INVESTMENT PICK 1727.00 24/12/2025 RECO PRICE RETURN TILL NOW 2297.30 133.02%</t>
@@ -60791,11 +60665,9 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1433" t="inlineStr"/>
       <c r="E1433" t="n">
         <v>4024.9</v>
       </c>
-      <c r="G1433" t="inlineStr"/>
       <c r="H1433" t="inlineStr">
         <is>
           <t>Sansera Engg 4024.90 INVESTMENT PICK 1727.00 24/12/2025 RECO PRICE RETURN TILL NOW 2297.90 133.06%</t>
@@ -60924,7 +60796,6 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="D1436" t="inlineStr"/>
       <c r="E1436" t="n">
         <v>535</v>
       </c>
@@ -61063,7 +60934,6 @@
       <c r="F1439" t="n">
         <v>999</v>
       </c>
-      <c r="G1439" t="inlineStr"/>
       <c r="H1439" t="inlineStr">
         <is>
           <t>सुमित बगडिया की राय Hindalco खरीदें PRICE 1017.40 TARGET 1040/1060 STOP LOSS 999</t>
@@ -61105,7 +60975,6 @@
       <c r="F1440" t="n">
         <v>999</v>
       </c>
-      <c r="G1440" t="inlineStr"/>
       <c r="H1440" t="inlineStr">
         <is>
           <t>सुमित बगडिया की राय Hindalco खरीदें PRICE 1017.40 TARGET 1040/1060 STOP LOSS 999</t>
@@ -61147,7 +61016,6 @@
       <c r="F1441" t="n">
         <v>4705</v>
       </c>
-      <c r="G1441" t="inlineStr"/>
       <c r="H1441" t="inlineStr">
         <is>
           <t>Data Patterns खरीदें PRICE 4745.30 TARGET 4800/4840 STOP LOSS 4705</t>
@@ -61229,7 +61097,6 @@
       <c r="E1443" t="n">
         <v>42000</v>
       </c>
-      <c r="G1443" t="inlineStr"/>
       <c r="H1443" t="inlineStr">
         <is>
           <t>सिटी
@@ -61315,7 +61182,6 @@
       <c r="E1445" t="n">
         <v>1280</v>
       </c>
-      <c r="G1445" t="inlineStr"/>
       <c r="H1445" t="inlineStr">
         <is>
           <t>Bharat Dynamics 1250.00 +8.30 HOLD लक्ष्य ₹1280</t>
@@ -61354,7 +61220,6 @@
       <c r="E1446" t="n">
         <v>1280</v>
       </c>
-      <c r="G1446" t="inlineStr"/>
       <c r="H1446" t="inlineStr">
         <is>
           <t>HDFC Life 539.00 5.80 1.09% Vol: 13.81 k PRE-OPEN BROKERAGE CALLS HOLD लक्ष्य ₹1280</t>
@@ -61396,7 +61261,6 @@
       <c r="F1447" t="n">
         <v>2425</v>
       </c>
-      <c r="G1447" t="inlineStr"/>
       <c r="H1447" t="inlineStr">
         <is>
           <t>MY CHOICE GLENMARK PHARMA B 2509 2425</t>
@@ -61435,7 +61299,6 @@
       <c r="E1448" t="n">
         <v>2509</v>
       </c>
-      <c r="G1448" t="inlineStr"/>
       <c r="H1448" t="inlineStr">
         <is>
           <t>MY CHOICE GLENMARK PHARMA B 2509</t>
@@ -61474,7 +61337,6 @@
       <c r="E1449" t="n">
         <v>3400</v>
       </c>
-      <c r="G1449" t="inlineStr"/>
       <c r="H1449" t="inlineStr">
         <is>
           <t>MY CHOICE MCX B 3400</t>
@@ -61513,7 +61375,6 @@
       <c r="F1450" t="n">
         <v>6</v>
       </c>
-      <c r="G1450" t="inlineStr"/>
       <c r="H1450" t="inlineStr">
         <is>
           <t>HDFC LIFE 540 CE B 16 6</t>
@@ -61552,7 +61413,6 @@
       <c r="E1451" t="n">
         <v>2588</v>
       </c>
-      <c r="G1451" t="inlineStr"/>
       <c r="H1451" t="inlineStr">
         <is>
           <t>PICK THE DAY Glenmark Pharma 2451.90 BUY TGT 2588</t>
@@ -61637,7 +61497,6 @@
       <c r="F1453" t="n">
         <v>1145</v>
       </c>
-      <c r="G1453" t="inlineStr"/>
       <c r="H1453" t="inlineStr">
         <is>
           <t>विश्वेश चौहान की राय
@@ -61684,7 +61543,6 @@
       <c r="F1454" t="n">
         <v>1145</v>
       </c>
-      <c r="G1454" t="inlineStr"/>
       <c r="H1454" t="inlineStr">
         <is>
           <t>विश्वेश चौहान की राय
@@ -61731,7 +61589,6 @@
       <c r="F1455" t="n">
         <v>12050</v>
       </c>
-      <c r="G1455" t="inlineStr"/>
       <c r="H1455" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Oracle Fin Fut SELL PRICE 11782.00 TARGET 11400/11000 STOP LOSS 12050</t>
@@ -61773,7 +61630,6 @@
       <c r="F1456" t="n">
         <v>12050</v>
       </c>
-      <c r="G1456" t="inlineStr"/>
       <c r="H1456" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Oracle Fin Fut SELL PRICE 11782.00 TARGET 11400/11000 STOP LOSS 12050</t>
@@ -61815,7 +61671,6 @@
       <c r="F1457" t="n">
         <v>2400</v>
       </c>
-      <c r="G1457" t="inlineStr"/>
       <c r="H1457" t="inlineStr">
         <is>
           <t>Glenmark Pharma BUY PRICE 2451.90 TARGET 2500/2530 STOP LOSS 2400</t>
@@ -61857,7 +61712,6 @@
       <c r="F1458" t="n">
         <v>2400</v>
       </c>
-      <c r="G1458" t="inlineStr"/>
       <c r="H1458" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Glenmark Pharma BUY PRICE 2451.90 TARGET 2500/2530 STOP LOSS 2400</t>
@@ -61896,7 +61750,6 @@
       <c r="E1459" t="n">
         <v>1220</v>
       </c>
-      <c r="G1459" t="inlineStr"/>
       <c r="H1459" t="inlineStr">
         <is>
           <t>PICK OF THE DAY
@@ -61940,7 +61793,6 @@
       <c r="E1460" t="n">
         <v>1250</v>
       </c>
-      <c r="G1460" t="inlineStr"/>
       <c r="H1460" t="inlineStr">
         <is>
           <t>PICK OF THE DAY
@@ -61987,7 +61839,6 @@
       <c r="F1461" t="n">
         <v>1105</v>
       </c>
-      <c r="G1461" t="inlineStr"/>
       <c r="H1461" t="inlineStr">
         <is>
           <t>विश्वेश चौहान की राय
@@ -62034,7 +61885,6 @@
       <c r="F1462" t="n">
         <v>3140</v>
       </c>
-      <c r="G1462" t="inlineStr"/>
       <c r="H1462" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Cartrade Tech BUY PRICE 3179.90 TARGET 3250/3280 STOP LOSS 3140</t>
@@ -62076,7 +61926,6 @@
       <c r="F1463" t="n">
         <v>3140</v>
       </c>
-      <c r="G1463" t="inlineStr"/>
       <c r="H1463" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Cartrade Tech BUY PRICE 3179.90 TARGET 3250/3280 STOP LOSS 3140</t>
@@ -62118,7 +61967,6 @@
       <c r="F1464" t="n">
         <v>930</v>
       </c>
-      <c r="G1464" t="inlineStr"/>
       <c r="H1464" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Jubilant Pharmova BUY PRICE 950.30 TARGET 990/1020 STOP LOSS 930</t>
@@ -62160,7 +62008,6 @@
       <c r="F1465" t="n">
         <v>930</v>
       </c>
-      <c r="G1465" t="inlineStr"/>
       <c r="H1465" t="inlineStr">
         <is>
           <t>PICK OF THE DAY Jubilant Pharmova BUY PRICE 950.30 TARGET 990/1020 STOP LOSS 930</t>
@@ -62202,7 +62049,6 @@
       <c r="F1466" t="n">
         <v>980</v>
       </c>
-      <c r="G1466" t="inlineStr"/>
       <c r="H1466" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -62249,7 +62095,6 @@
       <c r="F1467" t="n">
         <v>980</v>
       </c>
-      <c r="G1467" t="inlineStr"/>
       <c r="H1467" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -62296,7 +62141,6 @@
       <c r="F1468" t="n">
         <v>980</v>
       </c>
-      <c r="G1468" t="inlineStr"/>
       <c r="H1468" t="inlineStr">
         <is>
           <t>STOCK OF THE DAY
@@ -62343,7 +62187,6 @@
       <c r="F1469" t="n">
         <v>3298</v>
       </c>
-      <c r="G1469" t="inlineStr"/>
       <c r="H1469" t="inlineStr">
         <is>
           <t>MY CHOICE MCX B 3400 3298</t>
@@ -62385,7 +62228,6 @@
       <c r="F1470" t="n">
         <v>1951</v>
       </c>
-      <c r="G1470" t="inlineStr"/>
       <c r="H1470" t="inlineStr">
         <is>
           <t>CASH COROMANDEL INT B 2023 1951</t>
@@ -62424,7 +62266,6 @@
       <c r="E1471" t="n">
         <v>1910</v>
       </c>
-      <c r="G1471" t="inlineStr"/>
       <c r="H1471" t="inlineStr">
         <is>
           <t>INVESTMENT ASHOK LEYLAND B 1910 12M</t>
@@ -62463,7 +62304,6 @@
       <c r="E1472" t="n">
         <v>5100</v>
       </c>
-      <c r="G1472" t="inlineStr"/>
       <c r="H1472" t="inlineStr">
         <is>
           <t>FUNDA HAL B 5100 6 MONTH</t>
@@ -62505,7 +62345,6 @@
       <c r="F1473" t="n">
         <v>160</v>
       </c>
-      <c r="G1473" t="inlineStr"/>
       <c r="H1473" t="inlineStr">
         <is>
           <t>MY CHOICE Samvardhana Motherson खरीदें PRICE 162.00 TARGET 166 STOP LOSS 160</t>
@@ -62547,7 +62386,6 @@
       <c r="F1474" t="n">
         <v>2425</v>
       </c>
-      <c r="G1474" t="inlineStr"/>
       <c r="H1474" t="inlineStr">
         <is>
           <t>MY CHOICE Glenmark Pharma खरीदें PRICE 2451.90 TARGET 2509 STOP LOSS 2425</t>
@@ -62589,7 +62427,6 @@
       <c r="F1475" t="n">
         <v>400</v>
       </c>
-      <c r="G1475" t="inlineStr"/>
       <c r="H1475" t="inlineStr">
         <is>
           <t>MY CHOICE BEL खरीदें PRICE 404.00 TARGET 415 STOP LOSS 400</t>
@@ -62628,7 +62465,6 @@
       <c r="E1476" t="n">
         <v>415</v>
       </c>
-      <c r="G1476" t="inlineStr"/>
       <c r="H1476" t="inlineStr">
         <is>
           <t>MY CHOICE BEL PRICE 404.00 TARGET 415</t>
@@ -62667,7 +62503,6 @@
       <c r="E1477" t="n">
         <v>190</v>
       </c>
-      <c r="G1477" t="inlineStr"/>
       <c r="H1477" t="inlineStr">
         <is>
           <t>Ashok Leyland खरीदें PRICE 170.00 TARGET 190 DURATION 12 महीने</t>
@@ -62709,7 +62544,6 @@
       <c r="F1478" t="n">
         <v>22100</v>
       </c>
-      <c r="G1478" t="inlineStr"/>
       <c r="H1478" t="inlineStr">
         <is>
           <t>Shree Cement खरीदें PRICE 23365.00 TARGET 26000 STOP LOSS 22100</t>
@@ -62751,7 +62585,6 @@
       <c r="F1479" t="n">
         <v>1041</v>
       </c>
-      <c r="G1479" t="inlineStr"/>
       <c r="H1479" t="inlineStr">
         <is>
           <t>TECHNO PICK
@@ -62798,7 +62631,6 @@
       <c r="F1480" t="n">
         <v>6</v>
       </c>
-      <c r="G1480" t="inlineStr"/>
       <c r="H1480" t="inlineStr">
         <is>
           <t>BEST ऑप्शन HDFC Life 540 की कॉल खरीदें STOP LOSS 6 TARGET 16 HDFC Life 533.20 13.20</t>
@@ -62840,7 +62672,6 @@
       <c r="F1481" t="n">
         <v>1951</v>
       </c>
-      <c r="G1481" t="inlineStr"/>
       <c r="H1481" t="inlineStr">
         <is>
           <t>CASH का शेयर Coromandel Intl खरीदें PRICE 1974.60 TARGET 2023 STOP LOSS 1951</t>
@@ -62879,7 +62710,6 @@
       <c r="E1482" t="n">
         <v>478.3</v>
       </c>
-      <c r="G1482" t="inlineStr"/>
       <c r="H1482" t="inlineStr">
         <is>
           <t>पूजा के शेयर
@@ -62966,7 +62796,6 @@
       <c r="F1484" t="n">
         <v>181</v>
       </c>
-      <c r="G1484" t="inlineStr"/>
       <c r="H1484" t="inlineStr">
         <is>
           <t>अर्पित बेरीवाल की राय
@@ -63013,7 +62842,6 @@
       <c r="F1485" t="n">
         <v>9000</v>
       </c>
-      <c r="G1485" t="inlineStr"/>
       <c r="H1485" t="inlineStr">
         <is>
           <t>अर्पित बेरीवाल की राय
@@ -63057,7 +62885,6 @@
       <c r="E1486" t="n">
         <v>250</v>
       </c>
-      <c r="G1486" t="inlineStr"/>
       <c r="H1486" t="inlineStr">
         <is>
           <t>BROKERAGE CALLS
@@ -63100,7 +62927,6 @@
       <c r="E1487" t="n">
         <v>4954</v>
       </c>
-      <c r="G1487" t="inlineStr"/>
       <c r="H1487" t="inlineStr">
         <is>
           <t>BROKERAGE CALLS
@@ -63189,7 +63015,6 @@
       <c r="F1489" t="n">
         <v>8475</v>
       </c>
-      <c r="G1489" t="inlineStr"/>
       <c r="H1489" t="inlineStr">
         <is>
           <t>INTRADAY CALL Navin Fluorine BUY TARGET 8850 STOP LOSS 8475 Navin Fluorine 8603.50 0.54%</t>
@@ -63231,7 +63056,6 @@
       <c r="F1490" t="n">
         <v>360</v>
       </c>
-      <c r="G1490" t="inlineStr"/>
       <c r="H1490" t="inlineStr">
         <is>
           <t>POSITIONAL CALL M&amp;M Fin BUY TARGET 396 STOP LOSS 360 M&amp;M Fin 372.35 0.35%</t>
@@ -63248,8 +63072,3066 @@
         </is>
       </c>
     </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:22:42</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>RPSGVENT</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr"/>
+      <c r="E1491" t="n">
+        <v>950</v>
+      </c>
+      <c r="F1491" t="n">
+        <v>810</v>
+      </c>
+      <c r="G1491" t="inlineStr">
+        <is>
+          <t>Vikas Sethi</t>
+        </is>
+      </c>
+      <c r="H1491" t="inlineStr">
+        <is>
+          <t>विकास सेठी की राय RPSG Ventures @ 857 खरीदें STOP LOSS 810 TARGET 950 DURATION 4-8 महीने RPSG Ventures 873.45 6.64%</t>
+        </is>
+      </c>
+      <c r="I1491" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1491" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:15:00</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>ASAHIINDIA</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1492" t="n">
+        <v>953.5</v>
+      </c>
+      <c r="E1492" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F1492" t="n">
+        <v>870</v>
+      </c>
+      <c r="G1492" t="inlineStr">
+        <is>
+          <t>Vikas Sethi</t>
+        </is>
+      </c>
+      <c r="H1492" t="inlineStr">
+        <is>
+          <t>विकास सेठी की राय
+Asahi India Glass @950
+खरीदें
+STOP LOSS 870 | TARGET 1125 | DURATION 9-12 महीने
+Asahi India Glass 956.85 ▲ 0.13%</t>
+        </is>
+      </c>
+      <c r="I1492" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1492" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:03:00</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>GMDCLTD</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1493" t="n">
+        <v>579</v>
+      </c>
+      <c r="E1493" t="n">
+        <v>640</v>
+      </c>
+      <c r="F1493" t="n">
+        <v>550</v>
+      </c>
+      <c r="G1493" t="inlineStr"/>
+      <c r="H1493" t="inlineStr">
+        <is>
+          <t>Super KOOL MEHUL GMDC 579.00 10.15 BUY TGT 640 SL 550</t>
+        </is>
+      </c>
+      <c r="I1493" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1493" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:03:00</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1494" t="n">
+        <v>433.45</v>
+      </c>
+      <c r="E1494" t="n">
+        <v>445</v>
+      </c>
+      <c r="F1494" t="n">
+        <v>416</v>
+      </c>
+      <c r="G1494" t="inlineStr"/>
+      <c r="H1494" t="inlineStr">
+        <is>
+          <t>सुमित के सुपरहिट Coal India 433.30 13.05 BUY TGT 445 SL 416</t>
+        </is>
+      </c>
+      <c r="I1494" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1494" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:03:00</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1495" t="n">
+        <v>433.45</v>
+      </c>
+      <c r="E1495" t="n">
+        <v>445</v>
+      </c>
+      <c r="G1495" t="inlineStr"/>
+      <c r="H1495" t="inlineStr">
+        <is>
+          <t>Coal India 433.05 12.80 BUY TGT 445</t>
+        </is>
+      </c>
+      <c r="I1495" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1495" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:03:00</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1496" t="n">
+        <v>1034.5</v>
+      </c>
+      <c r="E1496" t="n">
+        <v>1055</v>
+      </c>
+      <c r="F1496" t="n">
+        <v>999</v>
+      </c>
+      <c r="G1496" t="inlineStr"/>
+      <c r="H1496" t="inlineStr">
+        <is>
+          <t>शुभ 'मंगला' शेयर Max Healthcare 1030.30 3.76% BUY TGT 1055 SL 999</t>
+        </is>
+      </c>
+      <c r="I1496" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1496" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:03:00</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>JSWENERGY</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1497" t="n">
+        <v>538.1</v>
+      </c>
+      <c r="E1497" t="n">
+        <v>560</v>
+      </c>
+      <c r="F1497" t="n">
+        <v>515</v>
+      </c>
+      <c r="G1497" t="inlineStr">
+        <is>
+          <t>Mehul</t>
+        </is>
+      </c>
+      <c r="H1497" t="inlineStr">
+        <is>
+          <t>Super KOOL MEHUL JSW Energy 538.20 11.80 BUY TGT 560 SL 515</t>
+        </is>
+      </c>
+      <c r="I1497" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1497" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:51:00</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1498" t="n">
+        <v>318.9</v>
+      </c>
+      <c r="E1498" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1498" t="inlineStr"/>
+      <c r="H1498" t="inlineStr">
+        <is>
+          <t>SID Eternal (Zomato) CMP 318.90 TARGET 400 25% ALLOCATION</t>
+        </is>
+      </c>
+      <c r="I1498" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1498" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:50:00</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>MEESHO</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1499" t="n">
+        <v>213.49</v>
+      </c>
+      <c r="E1499" t="n">
+        <v>230</v>
+      </c>
+      <c r="G1499" t="inlineStr"/>
+      <c r="H1499" t="inlineStr">
+        <is>
+          <t>'Gift Hamper' थीम Meesho CMP 213.50 TARGET 230 25% ALLOCATION</t>
+        </is>
+      </c>
+      <c r="I1499" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1499" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:37:03</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>SAMBHV</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr"/>
+      <c r="E1500" t="n">
+        <v>150</v>
+      </c>
+      <c r="G1500" t="inlineStr"/>
+      <c r="H1500" t="inlineStr">
+        <is>
+          <t>जैन साब के GEMS Sambhv Steel @ 130 खरीदें STOP LOSS -- TARGET 150 Sambhv Steel 131.55 ▲ 2.10%</t>
+        </is>
+      </c>
+      <c r="I1500" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1500" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:24:43</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>EIEL</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr"/>
+      <c r="E1501" t="n">
+        <v>192</v>
+      </c>
+      <c r="G1501" t="inlineStr"/>
+      <c r="H1501" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Enviro Infra 213.26 8.70% BUY TARGET HIT 192</t>
+        </is>
+      </c>
+      <c r="I1501" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1501" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:21:39</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>GRAPHITE</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr"/>
+      <c r="E1502" t="n">
+        <v>705</v>
+      </c>
+      <c r="G1502" t="inlineStr"/>
+      <c r="H1502" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Graphite India 806.90 72.65 BUY TARGET HIT 705</t>
+        </is>
+      </c>
+      <c r="I1502" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1502" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:22:00</t>
+        </is>
+      </c>
+      <c r="B1503" t="inlineStr">
+        <is>
+          <t>BIOCON</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1503" t="n">
+        <v>402.7</v>
+      </c>
+      <c r="E1503" t="n">
+        <v>807.05</v>
+      </c>
+      <c r="G1503" t="inlineStr"/>
+      <c r="H1503" t="inlineStr">
+        <is>
+          <t>Biocon 401.65 9.35 2.38% Vol: 2.3 m ▲ PICK OF THE DAY 807.05 TARGET HIT</t>
+        </is>
+      </c>
+      <c r="I1503" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1503" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:21:35</t>
+        </is>
+      </c>
+      <c r="B1504" t="inlineStr">
+        <is>
+          <t>GRAPHITE</t>
+        </is>
+      </c>
+      <c r="C1504" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1504" t="inlineStr"/>
+      <c r="E1504" t="n">
+        <v>760</v>
+      </c>
+      <c r="F1504" t="n">
+        <v>705</v>
+      </c>
+      <c r="G1504" t="inlineStr"/>
+      <c r="H1504" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY Graphite India 806.60 72.35 BUY TGT 760 SL 705</t>
+        </is>
+      </c>
+      <c r="I1504" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1504" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:21:29</t>
+        </is>
+      </c>
+      <c r="B1505" t="inlineStr">
+        <is>
+          <t>HEG-BE</t>
+        </is>
+      </c>
+      <c r="C1505" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1505" t="inlineStr"/>
+      <c r="E1505" t="n">
+        <v>252</v>
+      </c>
+      <c r="G1505" t="inlineStr"/>
+      <c r="H1505" t="inlineStr">
+        <is>
+          <t>मेहुल कोटारी HEG Ltd 263.95 2.07% BUY TARGET HIT 252</t>
+        </is>
+      </c>
+      <c r="I1505" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1505" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:22:00</t>
+        </is>
+      </c>
+      <c r="B1506" t="inlineStr">
+        <is>
+          <t>HEG-BE</t>
+        </is>
+      </c>
+      <c r="C1506" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1506" t="n">
+        <v>264.95</v>
+      </c>
+      <c r="E1506" t="n">
+        <v>265</v>
+      </c>
+      <c r="F1506" t="n">
+        <v>252</v>
+      </c>
+      <c r="G1506" t="inlineStr"/>
+      <c r="H1506" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY
+HEG Ltd
+263.95 5.35
+BUY
+TGT 265
+SL 252</t>
+        </is>
+      </c>
+      <c r="I1506" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1506" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:22:00</t>
+        </is>
+      </c>
+      <c r="B1507" t="inlineStr">
+        <is>
+          <t>JSWENERGY</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1507" t="n">
+        <v>533.6</v>
+      </c>
+      <c r="E1507" t="n">
+        <v>560</v>
+      </c>
+      <c r="F1507" t="n">
+        <v>515</v>
+      </c>
+      <c r="G1507" t="inlineStr"/>
+      <c r="H1507" t="inlineStr">
+        <is>
+          <t>Super Kool Menu
+JSW Energy
+खरीदें
+PRICE 532.75
+TARGET 560
+STOP LOSS 515</t>
+        </is>
+      </c>
+      <c r="I1507" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1507" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1508" t="inlineStr">
+        <is>
+          <t>BSE29SEP26</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1508" t="n">
+        <v>3305</v>
+      </c>
+      <c r="E1508" t="n">
+        <v>3300</v>
+      </c>
+      <c r="F1508" t="n">
+        <v>3460</v>
+      </c>
+      <c r="G1508" t="inlineStr"/>
+      <c r="H1508" t="inlineStr">
+        <is>
+          <t>STOCK OF THE DAY
+BSE Fut
+SELL
+PRICE ▶ 3403.20
+TARGET ▶ 3370, 3340, 3300
+STOP LOSS ▶ 3460</t>
+        </is>
+      </c>
+      <c r="I1508" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1508" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1509" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1509" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1509" t="n">
+        <v>237.8</v>
+      </c>
+      <c r="E1509" t="n">
+        <v>242</v>
+      </c>
+      <c r="F1509" t="n">
+        <v>230</v>
+      </c>
+      <c r="G1509" t="inlineStr"/>
+      <c r="H1509" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY ONGC 236.00 2.30 BUY TGT 242 SL 230</t>
+        </is>
+      </c>
+      <c r="I1509" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1509" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1510" t="inlineStr">
+        <is>
+          <t>BPCL29SEP26</t>
+        </is>
+      </c>
+      <c r="C1510" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1510" t="n">
+        <v>300.5</v>
+      </c>
+      <c r="E1510" t="n">
+        <v>287</v>
+      </c>
+      <c r="F1510" t="n">
+        <v>310</v>
+      </c>
+      <c r="G1510" t="inlineStr"/>
+      <c r="H1510" t="inlineStr">
+        <is>
+          <t>BPCL Fut SELL PRICE 303.60 TARGET 295/287 STOP LOSS 310</t>
+        </is>
+      </c>
+      <c r="I1510" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1510" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1511" t="inlineStr">
+        <is>
+          <t>BPCL29SEP26</t>
+        </is>
+      </c>
+      <c r="C1511" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1511" t="n">
+        <v>300.5</v>
+      </c>
+      <c r="E1511" t="n">
+        <v>295</v>
+      </c>
+      <c r="F1511" t="n">
+        <v>310</v>
+      </c>
+      <c r="G1511" t="inlineStr"/>
+      <c r="H1511" t="inlineStr">
+        <is>
+          <t>BPCL Fut SELL PRICE 303.60 TARGET 295/287 STOP LOSS 310</t>
+        </is>
+      </c>
+      <c r="I1511" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1511" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1512" t="inlineStr">
+        <is>
+          <t>AXISCADES</t>
+        </is>
+      </c>
+      <c r="C1512" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1512" t="n">
+        <v>1859</v>
+      </c>
+      <c r="E1512" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F1512" t="n">
+        <v>1779</v>
+      </c>
+      <c r="G1512" t="inlineStr"/>
+      <c r="H1512" t="inlineStr">
+        <is>
+          <t>Axiscades BUY PRICE 1848.60 TARGET 2000 STOP LOSS 1779</t>
+        </is>
+      </c>
+      <c r="I1512" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1512" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1513" t="inlineStr">
+        <is>
+          <t>HINDCOPPER</t>
+        </is>
+      </c>
+      <c r="C1513" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1513" t="n">
+        <v>539.4</v>
+      </c>
+      <c r="E1513" t="n">
+        <v>585</v>
+      </c>
+      <c r="F1513" t="n">
+        <v>510</v>
+      </c>
+      <c r="G1513" t="inlineStr"/>
+      <c r="H1513" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY
+Hind Copper
+BUY
+PRICE 532.85
+TARGET 570/585
+STOP LOSS 510</t>
+        </is>
+      </c>
+      <c r="I1513" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1513" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1514" t="inlineStr">
+        <is>
+          <t>HINDCOPPER</t>
+        </is>
+      </c>
+      <c r="C1514" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1514" t="n">
+        <v>539.35</v>
+      </c>
+      <c r="E1514" t="n">
+        <v>570</v>
+      </c>
+      <c r="F1514" t="n">
+        <v>510</v>
+      </c>
+      <c r="G1514" t="inlineStr"/>
+      <c r="H1514" t="inlineStr">
+        <is>
+          <t>PICK OF THE DAY
+Hind Copper
+BUY
+PRICE 532.85
+TARGET 570/585
+STOP LOSS 510</t>
+        </is>
+      </c>
+      <c r="I1514" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1514" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1515" t="inlineStr">
+        <is>
+          <t>RAYMONDLSL</t>
+        </is>
+      </c>
+      <c r="C1515" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1515" t="n">
+        <v>720</v>
+      </c>
+      <c r="E1515" t="n">
+        <v>725</v>
+      </c>
+      <c r="F1515" t="n">
+        <v>690</v>
+      </c>
+      <c r="G1515" t="inlineStr"/>
+      <c r="H1515" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह Raymond Lifestyle BUY PRICE 697 TARGET 705, 715, 725 STOP LOSS 690</t>
+        </is>
+      </c>
+      <c r="I1515" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1515" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1516" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV</t>
+        </is>
+      </c>
+      <c r="C1516" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1516" t="n">
+        <v>213.43</v>
+      </c>
+      <c r="E1516" t="n">
+        <v>215</v>
+      </c>
+      <c r="F1516" t="n">
+        <v>204</v>
+      </c>
+      <c r="G1516" t="inlineStr"/>
+      <c r="H1516" t="inlineStr">
+        <is>
+          <t>अनिल सिंघवी की सलाह
+Welspun Living
+BUY
+PRICE 208
+TARGET 210, 212, 215
+STOP LOSS 204</t>
+        </is>
+      </c>
+      <c r="I1516" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1516" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1517" t="inlineStr">
+        <is>
+          <t>FINCABLES</t>
+        </is>
+      </c>
+      <c r="C1517" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1517" t="n">
+        <v>1306</v>
+      </c>
+      <c r="E1517" t="n">
+        <v>1418</v>
+      </c>
+      <c r="G1517" t="inlineStr"/>
+      <c r="H1517" t="inlineStr">
+        <is>
+          <t>CALLS Finolex Cables 1302 BUY लक्ष्य ₹1418</t>
+        </is>
+      </c>
+      <c r="I1517" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1517" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:08</t>
+        </is>
+      </c>
+      <c r="B1518" t="inlineStr">
+        <is>
+          <t>JKLAKSHMI</t>
+        </is>
+      </c>
+      <c r="C1518" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1518" t="n">
+        <v>499.55</v>
+      </c>
+      <c r="E1518" t="n">
+        <v>1410</v>
+      </c>
+      <c r="G1518" t="inlineStr"/>
+      <c r="H1518" t="inlineStr">
+        <is>
+          <t>BROKERAGE CALLS BUY लक्ष्मी ₹1410</t>
+        </is>
+      </c>
+      <c r="I1518" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1518" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:03</t>
+        </is>
+      </c>
+      <c r="B1519" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C1519" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1519" t="n">
+        <v>3299.9</v>
+      </c>
+      <c r="E1519" t="n">
+        <v>2820</v>
+      </c>
+      <c r="G1519" t="inlineStr"/>
+      <c r="H1519" t="inlineStr">
+        <is>
+          <t>BROKERAGE CALLS
+BSE Ltd.
+3394.00 -52.20
+UNDER PERFORM
+लक्ष्य ₹2820</t>
+        </is>
+      </c>
+      <c r="I1519" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1519" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1520" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV</t>
+        </is>
+      </c>
+      <c r="C1520" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1520" t="n">
+        <v>213.43</v>
+      </c>
+      <c r="E1520" t="n">
+        <v>260</v>
+      </c>
+      <c r="G1520" t="inlineStr">
+        <is>
+          <t>Jefferies</t>
+        </is>
+      </c>
+      <c r="H1520" t="inlineStr">
+        <is>
+          <t>जेफरीज Welspun Living 207.87 -4.08 BUY लक्ष्य ₹260</t>
+        </is>
+      </c>
+      <c r="I1520" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1520" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1521" t="inlineStr">
+        <is>
+          <t>RAYMONDLSL</t>
+        </is>
+      </c>
+      <c r="C1521" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1521" t="n">
+        <v>720</v>
+      </c>
+      <c r="E1521" t="n">
+        <v>900</v>
+      </c>
+      <c r="G1521" t="inlineStr">
+        <is>
+          <t>Jefferies</t>
+        </is>
+      </c>
+      <c r="H1521" t="inlineStr">
+        <is>
+          <t>जेफरीज Raymond Lifestyle 696.85 +23.95 BUY लक्ष्य ₹900</t>
+        </is>
+      </c>
+      <c r="I1521" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1521" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1522" t="inlineStr">
+        <is>
+          <t>BPCL29SEP26</t>
+        </is>
+      </c>
+      <c r="C1522" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1522" t="n">
+        <v>301.95</v>
+      </c>
+      <c r="E1522" t="n">
+        <v>295</v>
+      </c>
+      <c r="F1522" t="n">
+        <v>307</v>
+      </c>
+      <c r="G1522" t="inlineStr"/>
+      <c r="H1522" t="inlineStr">
+        <is>
+          <t>MY CHOICE BPCL FUT S 295 307</t>
+        </is>
+      </c>
+      <c r="I1522" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1522" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:01</t>
+        </is>
+      </c>
+      <c r="B1523" t="inlineStr">
+        <is>
+          <t>ASIANPAINT29SEP26</t>
+        </is>
+      </c>
+      <c r="C1523" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1523" t="n">
+        <v>2470</v>
+      </c>
+      <c r="E1523" t="n">
+        <v>2430</v>
+      </c>
+      <c r="F1523" t="n">
+        <v>2505</v>
+      </c>
+      <c r="G1523" t="inlineStr"/>
+      <c r="H1523" t="inlineStr">
+        <is>
+          <t>MY CHOICE ASIAN PAINTS FUT S 2430 2505</t>
+        </is>
+      </c>
+      <c r="I1523" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1523" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1524" t="inlineStr">
+        <is>
+          <t>HINDPETRO29SEP26</t>
+        </is>
+      </c>
+      <c r="C1524" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1524" t="n">
+        <v>347</v>
+      </c>
+      <c r="E1524" t="n">
+        <v>339</v>
+      </c>
+      <c r="F1524" t="n">
+        <v>350</v>
+      </c>
+      <c r="G1524" t="inlineStr"/>
+      <c r="H1524" t="inlineStr">
+        <is>
+          <t>MY CHOICE HPCL FUT S 339 350</t>
+        </is>
+      </c>
+      <c r="I1524" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1524" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1525" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV</t>
+        </is>
+      </c>
+      <c r="C1525" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1525" t="n">
+        <v>213.43</v>
+      </c>
+      <c r="E1525" t="n">
+        <v>230</v>
+      </c>
+      <c r="G1525" t="inlineStr"/>
+      <c r="H1525" t="inlineStr">
+        <is>
+          <t>INVESTMENT WELSPUN LIVING B 230 12 MONTH</t>
+        </is>
+      </c>
+      <c r="I1525" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1525" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1526" t="inlineStr">
+        <is>
+          <t>FINCABLES</t>
+        </is>
+      </c>
+      <c r="C1526" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1526" t="n">
+        <v>1306</v>
+      </c>
+      <c r="E1526" t="n">
+        <v>1328</v>
+      </c>
+      <c r="F1526" t="n">
+        <v>1289</v>
+      </c>
+      <c r="G1526" t="inlineStr"/>
+      <c r="H1526" t="inlineStr">
+        <is>
+          <t>NEWS IMPACT FINOLEX CABLES B 1328 1289</t>
+        </is>
+      </c>
+      <c r="I1526" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1526" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1527" t="inlineStr">
+        <is>
+          <t>HINDCOPPER</t>
+        </is>
+      </c>
+      <c r="C1527" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1527" t="n">
+        <v>538</v>
+      </c>
+      <c r="E1527" t="n">
+        <v>545</v>
+      </c>
+      <c r="F1527" t="n">
+        <v>527</v>
+      </c>
+      <c r="G1527" t="inlineStr"/>
+      <c r="H1527" t="inlineStr">
+        <is>
+          <t>CASH HINDUSTAN COPPER B 545 527</t>
+        </is>
+      </c>
+      <c r="I1527" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1527" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1528" t="inlineStr">
+        <is>
+          <t>BEML</t>
+        </is>
+      </c>
+      <c r="C1528" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1528" t="n">
+        <v>2105</v>
+      </c>
+      <c r="E1528" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G1528" t="inlineStr"/>
+      <c r="H1528" t="inlineStr">
+        <is>
+          <t>FUNDA BEML B 2200 6 MONTHS</t>
+        </is>
+      </c>
+      <c r="I1528" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1528" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1529" t="inlineStr">
+        <is>
+          <t>NATIONALUM29SEP26</t>
+        </is>
+      </c>
+      <c r="C1529" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1529" t="n">
+        <v>373.3</v>
+      </c>
+      <c r="E1529" t="n">
+        <v>380</v>
+      </c>
+      <c r="F1529" t="n">
+        <v>367</v>
+      </c>
+      <c r="G1529" t="inlineStr"/>
+      <c r="H1529" t="inlineStr">
+        <is>
+          <t>FUTURE NALCO FUT B 380 367</t>
+        </is>
+      </c>
+      <c r="I1529" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1529" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1530" t="inlineStr">
+        <is>
+          <t>HDFCBANK29SEP26</t>
+        </is>
+      </c>
+      <c r="C1530" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1530" t="n">
+        <v>702.9</v>
+      </c>
+      <c r="E1530" t="n">
+        <v>694</v>
+      </c>
+      <c r="F1530" t="n">
+        <v>715</v>
+      </c>
+      <c r="G1530" t="inlineStr"/>
+      <c r="H1530" t="inlineStr">
+        <is>
+          <t>TECHNO HDFC BANK FUT S 694 715</t>
+        </is>
+      </c>
+      <c r="I1530" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1530" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1531" t="inlineStr">
+        <is>
+          <t>NLCINDIA</t>
+        </is>
+      </c>
+      <c r="C1531" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1531" t="n">
+        <v>273.6</v>
+      </c>
+      <c r="E1531" t="n">
+        <v>282</v>
+      </c>
+      <c r="F1531" t="n">
+        <v>268</v>
+      </c>
+      <c r="G1531" t="inlineStr"/>
+      <c r="H1531" t="inlineStr">
+        <is>
+          <t>CASH NLC INDIA B 282 268</t>
+        </is>
+      </c>
+      <c r="I1531" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1531" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1532" t="inlineStr">
+        <is>
+          <t>HAL29SEP26</t>
+        </is>
+      </c>
+      <c r="C1532" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1532" t="n">
+        <v>5063.8</v>
+      </c>
+      <c r="E1532" t="n">
+        <v>5180</v>
+      </c>
+      <c r="F1532" t="n">
+        <v>4981</v>
+      </c>
+      <c r="G1532" t="inlineStr"/>
+      <c r="H1532" t="inlineStr">
+        <is>
+          <t>FUTURE HAL FUT B 5180 4981</t>
+        </is>
+      </c>
+      <c r="I1532" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1532" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1533" t="inlineStr">
+        <is>
+          <t>BPCL29SEP26</t>
+        </is>
+      </c>
+      <c r="C1533" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1533" t="n">
+        <v>300.5</v>
+      </c>
+      <c r="E1533" t="n">
+        <v>295</v>
+      </c>
+      <c r="F1533" t="n">
+        <v>307</v>
+      </c>
+      <c r="G1533" t="inlineStr"/>
+      <c r="H1533" t="inlineStr">
+        <is>
+          <t>MY CHOICE BPCL Fut बेचें PRICE 303.60 TARGET 295 STOP LOSS 307</t>
+        </is>
+      </c>
+      <c r="I1533" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1533" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:01</t>
+        </is>
+      </c>
+      <c r="B1534" t="inlineStr">
+        <is>
+          <t>ASIANPAINT29SEP26</t>
+        </is>
+      </c>
+      <c r="C1534" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1534" t="n">
+        <v>2470</v>
+      </c>
+      <c r="E1534" t="n">
+        <v>2430</v>
+      </c>
+      <c r="F1534" t="n">
+        <v>2505</v>
+      </c>
+      <c r="G1534" t="inlineStr"/>
+      <c r="H1534" t="inlineStr">
+        <is>
+          <t>पूजा के शेयर
+Asian Paints Fut
+बेचें
+PRICE 2499.50
+TARGET 2430
+STOP LOSS 2505</t>
+        </is>
+      </c>
+      <c r="I1534" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1534" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1535" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1535" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1535" t="n">
+        <v>237.8</v>
+      </c>
+      <c r="E1535" t="n">
+        <v>241</v>
+      </c>
+      <c r="F1535" t="n">
+        <v>233.5</v>
+      </c>
+      <c r="G1535" t="inlineStr"/>
+      <c r="H1535" t="inlineStr">
+        <is>
+          <t>MY CHOICE ONGC खरीदें PRICE 236.00 TARGET 241 STOP LOSS 233.5</t>
+        </is>
+      </c>
+      <c r="I1535" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1535" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1536" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1536" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1536" t="n">
+        <v>237.8</v>
+      </c>
+      <c r="E1536" t="n">
+        <v>241</v>
+      </c>
+      <c r="G1536" t="inlineStr"/>
+      <c r="H1536" t="inlineStr">
+        <is>
+          <t>MY CHOICE ONGC PRICE 236.00 TARGET 241</t>
+        </is>
+      </c>
+      <c r="I1536" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1536" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1537" t="inlineStr">
+        <is>
+          <t>OIL</t>
+        </is>
+      </c>
+      <c r="C1537" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1537" t="n">
+        <v>498</v>
+      </c>
+      <c r="E1537" t="n">
+        <v>506.5</v>
+      </c>
+      <c r="F1537" t="n">
+        <v>488</v>
+      </c>
+      <c r="G1537" t="inlineStr"/>
+      <c r="H1537" t="inlineStr">
+        <is>
+          <t>नेहा के शेयर
+Oil India
+खरीदें
+PRICE ▶ 495.40
+TARGET ▶ 506.5
+STOP LOSS ▶ 488</t>
+        </is>
+      </c>
+      <c r="I1537" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1537" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1538" t="inlineStr">
+        <is>
+          <t>EIEL</t>
+        </is>
+      </c>
+      <c r="C1538" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1538" t="n">
+        <v>205.39</v>
+      </c>
+      <c r="E1538" t="n">
+        <v>206</v>
+      </c>
+      <c r="F1538" t="n">
+        <v>191</v>
+      </c>
+      <c r="G1538" t="inlineStr"/>
+      <c r="H1538" t="inlineStr">
+        <is>
+          <t>खबर के दम पर
+Enviro Infra
+खरीदें
+PRICE ▶ 196.20
+TARGET ▶ 206
+STOP LOSS ▶ 191</t>
+        </is>
+      </c>
+      <c r="I1538" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1538" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1539" t="inlineStr">
+        <is>
+          <t>FINCABLES</t>
+        </is>
+      </c>
+      <c r="C1539" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1539" t="n">
+        <v>1306</v>
+      </c>
+      <c r="E1539" t="n">
+        <v>1328</v>
+      </c>
+      <c r="F1539" t="n">
+        <v>1289</v>
+      </c>
+      <c r="G1539" t="inlineStr"/>
+      <c r="H1539" t="inlineStr">
+        <is>
+          <t>खबर के दम पर Finolex Cables खरीदें PRICE 1302.30 TARGET 1328 STOP LOSS 1289 STOCK OF THE DAY 8:25 AM 9AM</t>
+        </is>
+      </c>
+      <c r="I1539" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1539" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1540" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV</t>
+        </is>
+      </c>
+      <c r="C1540" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1540" t="n">
+        <v>213.43</v>
+      </c>
+      <c r="E1540" t="n">
+        <v>230</v>
+      </c>
+      <c r="G1540" t="inlineStr"/>
+      <c r="H1540" t="inlineStr">
+        <is>
+          <t>पूजा के शेयर Welspun Living खरीदें PRICE 207.87 TARGET 230 DURATION 12 महीने</t>
+        </is>
+      </c>
+      <c r="I1540" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1540" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:07</t>
+        </is>
+      </c>
+      <c r="B1541" t="inlineStr">
+        <is>
+          <t>GNA</t>
+        </is>
+      </c>
+      <c r="C1541" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1541" t="n">
+        <v>556</v>
+      </c>
+      <c r="E1541" t="n">
+        <v>700</v>
+      </c>
+      <c r="F1541" t="n">
+        <v>490</v>
+      </c>
+      <c r="G1541" t="inlineStr"/>
+      <c r="H1541" t="inlineStr">
+        <is>
+          <t>नेहा के शेयर
+GNA Axles
+खरीदें
+PRICE ▶ 553.40
+TARGET ▶ 700
+STOP LOSS ▶ 490</t>
+        </is>
+      </c>
+      <c r="I1541" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1541" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:01</t>
+        </is>
+      </c>
+      <c r="B1542" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="C1542" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1542" t="n">
+        <v>1013.9</v>
+      </c>
+      <c r="E1542" t="n">
+        <v>1025</v>
+      </c>
+      <c r="F1542" t="n">
+        <v>990</v>
+      </c>
+      <c r="G1542" t="inlineStr"/>
+      <c r="H1542" t="inlineStr">
+        <is>
+          <t>नेहा के शेयर Hindalco खरीदें PRICE 1009.00 TARGET 1025 STOP LOSS 990</t>
+        </is>
+      </c>
+      <c r="I1542" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1542" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:01</t>
+        </is>
+      </c>
+      <c r="B1543" t="inlineStr">
+        <is>
+          <t>BEML</t>
+        </is>
+      </c>
+      <c r="C1543" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1543" t="n">
+        <v>2105.8</v>
+      </c>
+      <c r="E1543" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G1543" t="inlineStr"/>
+      <c r="H1543" t="inlineStr">
+        <is>
+          <t>पूजा के शेयर
+BEML
+खरीदें
+PRICE ▶ 2105.60
+TARGET ▶ 2200
+DURATION ▶ 6 महीने</t>
+        </is>
+      </c>
+      <c r="I1543" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1543" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1544" t="inlineStr">
+        <is>
+          <t>INDIGO500029SEP26CE</t>
+        </is>
+      </c>
+      <c r="C1544" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1544" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="E1544" t="n">
+        <v>250</v>
+      </c>
+      <c r="F1544" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1544" t="inlineStr"/>
+      <c r="H1544" t="inlineStr">
+        <is>
+          <t>BEST ऑप्शन Interglobe Aviation 5000 की पुट @119.35 खरीदें STOP LOSS 60 TARGET 250</t>
+        </is>
+      </c>
+      <c r="I1544" t="inlineStr">
+        <is>
+          <t>660334625662a7f64ae8911d</t>
+        </is>
+      </c>
+      <c r="J1544" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1545" t="inlineStr">
+        <is>
+          <t>HDFCBANK29SEP26</t>
+        </is>
+      </c>
+      <c r="C1545" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D1545" t="n">
+        <v>702.9</v>
+      </c>
+      <c r="E1545" t="n">
+        <v>694</v>
+      </c>
+      <c r="F1545" t="n">
+        <v>715</v>
+      </c>
+      <c r="G1545" t="inlineStr"/>
+      <c r="H1545" t="inlineStr">
+        <is>
+          <t>TECHNO PICK
+HDFC Bank Fut
+बेचें
+PRICE ▶ 708.80
+TARGET ▶ 694
+STOP LOSS ▶ 715</t>
+        </is>
+      </c>
+      <c r="I1545" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1545" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1546" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="C1546" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1546" t="n">
+        <v>595</v>
+      </c>
+      <c r="E1546" t="n">
+        <v>621</v>
+      </c>
+      <c r="F1546" t="n">
+        <v>580</v>
+      </c>
+      <c r="G1546" t="inlineStr"/>
+      <c r="H1546" t="inlineStr">
+        <is>
+          <t>TECHNO PICK
+Hindustan Zinc
+खरीदें
+PRICE ▶ 595.50
+TARGET ▶ 621
+STOP LOSS ▶ 580</t>
+        </is>
+      </c>
+      <c r="I1546" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1546" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1547" t="inlineStr">
+        <is>
+          <t>AXISBANK124029SEP26PE</t>
+        </is>
+      </c>
+      <c r="C1547" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1547" t="n">
+        <v>18</v>
+      </c>
+      <c r="E1547" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1547" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1547" t="inlineStr"/>
+      <c r="H1547" t="inlineStr">
+        <is>
+          <t>नेहा के शेयर Axis Bank 1240 की पुट @ 24.8 खरीदें STOP LOSS 12 TARGET 50 Axis Bank 1244.90 1.67%</t>
+        </is>
+      </c>
+      <c r="I1547" t="inlineStr">
+        <is>
+          <t>660334625662a7f64ae8911d</t>
+        </is>
+      </c>
+      <c r="J1547" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1548" t="inlineStr">
+        <is>
+          <t>AXISBANK124029SEP26CE</t>
+        </is>
+      </c>
+      <c r="C1548" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1548" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E1548" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1548" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1548" t="inlineStr"/>
+      <c r="H1548" t="inlineStr">
+        <is>
+          <t>Axis Bank 1240 की पुट @ 24.8 खरीदें STOP LOSS 12 TARGET 50 Axis Bank 1244.90 1.67%</t>
+        </is>
+      </c>
+      <c r="I1548" t="inlineStr">
+        <is>
+          <t>660334625662a7f64ae8911d</t>
+        </is>
+      </c>
+      <c r="J1548" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1549" t="inlineStr">
+        <is>
+          <t>NATIONALUM29SEP26</t>
+        </is>
+      </c>
+      <c r="C1549" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1549" t="n">
+        <v>373.05</v>
+      </c>
+      <c r="E1549" t="n">
+        <v>380</v>
+      </c>
+      <c r="F1549" t="n">
+        <v>367</v>
+      </c>
+      <c r="G1549" t="inlineStr"/>
+      <c r="H1549" t="inlineStr">
+        <is>
+          <t>आज का FUTURE
+NALCO Fut
+खरीदें
+PRICE → 370.35
+TARGET → 380
+STOP LOSS → 367</t>
+        </is>
+      </c>
+      <c r="I1549" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1549" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1550" t="inlineStr">
+        <is>
+          <t>HAL29SEP26</t>
+        </is>
+      </c>
+      <c r="C1550" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1550" t="n">
+        <v>5063.8</v>
+      </c>
+      <c r="E1550" t="n">
+        <v>5180</v>
+      </c>
+      <c r="F1550" t="n">
+        <v>4981</v>
+      </c>
+      <c r="G1550" t="inlineStr"/>
+      <c r="H1550" t="inlineStr">
+        <is>
+          <t>नेहा के शेयर
+HAL Fut
+खरीदें
+PRICE ▸ 5063.80
+TARGET ▸ 5180
+STOP LOSS ▸ 4981</t>
+        </is>
+      </c>
+      <c r="I1550" t="inlineStr">
+        <is>
+          <t>660334275662a7f64ae8911c</t>
+        </is>
+      </c>
+      <c r="J1550" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:03</t>
+        </is>
+      </c>
+      <c r="B1551" t="inlineStr">
+        <is>
+          <t>NLCINDIA</t>
+        </is>
+      </c>
+      <c r="C1551" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1551" t="n">
+        <v>274.7</v>
+      </c>
+      <c r="E1551" t="n">
+        <v>282</v>
+      </c>
+      <c r="F1551" t="n">
+        <v>268</v>
+      </c>
+      <c r="G1551" t="inlineStr"/>
+      <c r="H1551" t="inlineStr">
+        <is>
+          <t>CASH का शेयर
+NLC India
+खरीदें
+PRICE ▶ 272.25
+TARGET ▶ 282
+STOP LOSS ▶ 268</t>
+        </is>
+      </c>
+      <c r="I1551" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1551" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:03</t>
+        </is>
+      </c>
+      <c r="B1552" t="inlineStr">
+        <is>
+          <t>NLCINDIA</t>
+        </is>
+      </c>
+      <c r="C1552" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1552" t="n">
+        <v>274.7</v>
+      </c>
+      <c r="E1552" t="n">
+        <v>282</v>
+      </c>
+      <c r="G1552" t="inlineStr"/>
+      <c r="H1552" t="inlineStr">
+        <is>
+          <t>CASH का शेयर
+NLC India
+PRICE 272.25
+TARGET 282</t>
+        </is>
+      </c>
+      <c r="I1552" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1552" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1553" t="inlineStr">
+        <is>
+          <t>HINDCOPPER</t>
+        </is>
+      </c>
+      <c r="C1553" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1553" t="n">
+        <v>539.35</v>
+      </c>
+      <c r="E1553" t="n">
+        <v>545</v>
+      </c>
+      <c r="F1553" t="n">
+        <v>527</v>
+      </c>
+      <c r="G1553" t="inlineStr"/>
+      <c r="H1553" t="inlineStr">
+        <is>
+          <t>CASH का शेयर Hind Copper खरीदें PRICE 532.85 TARGET 545 STOP LOSS 527</t>
+        </is>
+      </c>
+      <c r="I1553" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1553" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1554" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV</t>
+        </is>
+      </c>
+      <c r="C1554" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1554" t="n">
+        <v>214.22</v>
+      </c>
+      <c r="E1554" t="n">
+        <v>260</v>
+      </c>
+      <c r="G1554" t="inlineStr"/>
+      <c r="H1554" t="inlineStr">
+        <is>
+          <t>Welspun Living BUY 260</t>
+        </is>
+      </c>
+      <c r="I1554" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1554" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1555" t="inlineStr">
+        <is>
+          <t>RAYMONDLSL</t>
+        </is>
+      </c>
+      <c r="C1555" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1555" t="n">
+        <v>720</v>
+      </c>
+      <c r="E1555" t="n">
+        <v>900</v>
+      </c>
+      <c r="G1555" t="inlineStr"/>
+      <c r="H1555" t="inlineStr">
+        <is>
+          <t>Raymond Lifestyle BUY 900</t>
+        </is>
+      </c>
+      <c r="I1555" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1555" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:01</t>
+        </is>
+      </c>
+      <c r="B1556" t="inlineStr">
+        <is>
+          <t>LICHSGFIN</t>
+        </is>
+      </c>
+      <c r="C1556" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1556" t="n">
+        <v>560</v>
+      </c>
+      <c r="E1556" t="n">
+        <v>595</v>
+      </c>
+      <c r="F1556" t="n">
+        <v>548</v>
+      </c>
+      <c r="G1556" t="inlineStr"/>
+      <c r="H1556" t="inlineStr">
+        <is>
+          <t>TRADING CALL LIC Hsg Fin खरीदें PRICE 563.00 TARGET 585/595 STOP LOSS 548</t>
+        </is>
+      </c>
+      <c r="I1556" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1556" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:01</t>
+        </is>
+      </c>
+      <c r="B1557" t="inlineStr">
+        <is>
+          <t>LICHSGFIN</t>
+        </is>
+      </c>
+      <c r="C1557" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1557" t="n">
+        <v>560</v>
+      </c>
+      <c r="E1557" t="n">
+        <v>585</v>
+      </c>
+      <c r="F1557" t="n">
+        <v>548</v>
+      </c>
+      <c r="G1557" t="inlineStr"/>
+      <c r="H1557" t="inlineStr">
+        <is>
+          <t>TRADING CALL LIC Hsg Fin खरीदें PRICE 563.00 TARGET 585/595 STOP LOSS 548</t>
+        </is>
+      </c>
+      <c r="I1557" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1557" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1558" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="C1558" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1558" t="n">
+        <v>411.75</v>
+      </c>
+      <c r="E1558" t="n">
+        <v>430</v>
+      </c>
+      <c r="F1558" t="n">
+        <v>404</v>
+      </c>
+      <c r="G1558" t="inlineStr"/>
+      <c r="H1558" t="inlineStr">
+        <is>
+          <t>TRADING CALL BEL खरीदें PRICE 410.55 TARGET 425/430 STOP LOSS 404</t>
+        </is>
+      </c>
+      <c r="I1558" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1558" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1559" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="C1559" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1559" t="n">
+        <v>412</v>
+      </c>
+      <c r="E1559" t="n">
+        <v>425</v>
+      </c>
+      <c r="F1559" t="n">
+        <v>404</v>
+      </c>
+      <c r="G1559" t="inlineStr"/>
+      <c r="H1559" t="inlineStr">
+        <is>
+          <t>TRADING CALL BEL खरीदें PRICE 410.55 TARGET 425/430 STOP LOSS 404</t>
+        </is>
+      </c>
+      <c r="I1559" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1559" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1560" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="C1560" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1560" t="n">
+        <v>5047.7</v>
+      </c>
+      <c r="E1560" t="n">
+        <v>6175</v>
+      </c>
+      <c r="G1560" t="inlineStr"/>
+      <c r="H1560" t="inlineStr">
+        <is>
+          <t>सिटी HAL 5031.10 +175.90 BUY लक्ष्य ₹6175</t>
+        </is>
+      </c>
+      <c r="I1560" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1560" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:00</t>
+        </is>
+      </c>
+      <c r="B1561" t="inlineStr">
+        <is>
+          <t>FINCABLES</t>
+        </is>
+      </c>
+      <c r="C1561" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1561" t="n">
+        <v>1319.9</v>
+      </c>
+      <c r="E1561" t="n">
+        <v>1410</v>
+      </c>
+      <c r="G1561" t="inlineStr">
+        <is>
+          <t>Jefferies</t>
+        </is>
+      </c>
+      <c r="H1561" t="inlineStr">
+        <is>
+          <t>जेफरीज Finolex Cables 1302.30 +75.30 BUY लक्ष्य ₹1410</t>
+        </is>
+      </c>
+      <c r="I1561" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1561" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" t="inlineStr">
+        <is>
+          <t>2026-09-09 09:15:02</t>
+        </is>
+      </c>
+      <c r="B1562" t="inlineStr">
+        <is>
+          <t>NELCO</t>
+        </is>
+      </c>
+      <c r="C1562" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D1562" t="n">
+        <v>976.1</v>
+      </c>
+      <c r="E1562" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F1562" t="n">
+        <v>910</v>
+      </c>
+      <c r="G1562" t="inlineStr"/>
+      <c r="H1562" t="inlineStr">
+        <is>
+          <t>POSITIONAL CALL NELCO BUY TARGET 1070 STOP LOSS 910 NELCO 973.10 ▲ 39.90</t>
+        </is>
+      </c>
+      <c r="I1562" t="inlineStr">
+        <is>
+          <t>660333e45662a7f64ae8911b</t>
+        </is>
+      </c>
+      <c r="J1562" t="inlineStr">
+        <is>
+          <t>https://www.zeebusinesslive.com/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1490"/>
+  <autoFilter ref="A1:J1562"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>